<commit_message>
Add SOH report for 2026-10-22
</commit_message>
<xml_diff>
--- a/reports/SOH_22_10_2026.xlsx
+++ b/reports/SOH_22_10_2026.xlsx
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>1523</v>
+        <v>1503</v>
       </c>
       <c r="E140" s="3" t="n">
         <v>7845</v>
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="D255" s="2" t="n">
-        <v>788</v>
+        <v>776</v>
       </c>
       <c r="E255" s="3" t="n">
         <v>11491</v>
@@ -8421,7 +8421,7 @@
         </is>
       </c>
       <c r="D289" s="2" t="n">
-        <v>1094</v>
+        <v>1070</v>
       </c>
       <c r="E289" s="3" t="n">
         <v>7347</v>
@@ -8449,7 +8449,7 @@
         </is>
       </c>
       <c r="D290" s="2" t="n">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="E290" s="3" t="n">
         <v>8018</v>
@@ -9345,7 +9345,7 @@
         </is>
       </c>
       <c r="D322" s="2" t="n">
-        <v>591</v>
+        <v>567</v>
       </c>
       <c r="E322" s="3" t="n">
         <v>11822</v>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
       <c r="D323" s="2" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E323" s="3" t="n">
         <v>16171</v>
@@ -9794,7 +9794,7 @@
         </is>
       </c>
       <c r="D338" s="2" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E338" s="3" t="n">
         <v>5000</v>
@@ -9850,7 +9850,7 @@
         </is>
       </c>
       <c r="D340" s="2" t="n">
-        <v>-189</v>
+        <v>-113</v>
       </c>
       <c r="E340" s="3" t="n">
         <v>2500</v>
@@ -9962,7 +9962,7 @@
         </is>
       </c>
       <c r="D344" s="2" t="n">
-        <v>1170</v>
+        <v>1155</v>
       </c>
       <c r="E344" s="3" t="n">
         <v>10170</v>
@@ -10074,7 +10074,7 @@
         </is>
       </c>
       <c r="D348" s="2" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E348" s="3" t="n">
         <v>6251</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="D357" s="2" t="n">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="E357" s="3" t="n">
         <v>9468</v>
@@ -10578,7 +10578,7 @@
         </is>
       </c>
       <c r="D366" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E366" s="3" t="n">
         <v>16261</v>
@@ -13126,7 +13126,7 @@
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="E457" s="3" t="n">
         <v>8856</v>
@@ -13154,7 +13154,7 @@
         </is>
       </c>
       <c r="D458" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E458" s="3" t="n">
         <v>8856</v>
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="D459" s="2" t="n">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="E459" s="3" t="n">
         <v>8855.5</v>
@@ -13210,7 +13210,7 @@
         </is>
       </c>
       <c r="D460" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="E460" s="3" t="n">
         <v>8855.5</v>
@@ -13378,7 +13378,7 @@
         </is>
       </c>
       <c r="D466" s="2" t="n">
-        <v>662</v>
+        <v>642</v>
       </c>
       <c r="E466" s="3" t="n">
         <v>9621</v>
@@ -14540,24 +14540,24 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>9333527033208</t>
+          <t>9333527500861</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>SP0055</t>
+          <t>IL0303</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>COPY PAPER NEON 30pk A4</t>
+          <t>CORDLESS LIGHT BULB PORTABLE</t>
         </is>
       </c>
       <c r="D508" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E508" s="3" t="n">
-        <v>5652</v>
+        <v>17061</v>
       </c>
       <c r="F508" t="inlineStr">
         <is>
@@ -14568,24 +14568,24 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>9333527500861</t>
+          <t>9333527022059</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>IL0303</t>
+          <t>AG0128</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>CORDLESS LIGHT BULB PORTABLE</t>
+          <t>COSMETIC APPLIQUE TIPS 12PK 2ASST</t>
         </is>
       </c>
       <c r="D509" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E509" s="3" t="n">
-        <v>17061</v>
+        <v>6001</v>
       </c>
       <c r="F509" t="inlineStr">
         <is>
@@ -14596,24 +14596,24 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>9333527022059</t>
+          <t>9333527429872</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>AG0128</t>
+          <t>AG2086</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>COSMETIC APPLIQUE TIPS 12PK 2ASST</t>
+          <t>COSMETIC BAGS PK3 3 ASST</t>
         </is>
       </c>
       <c r="D510" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E510" s="3" t="n">
-        <v>6001</v>
+        <v>38243</v>
       </c>
       <c r="F510" t="inlineStr">
         <is>
@@ -14624,24 +14624,24 @@
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>9333527429872</t>
+          <t>9333527429797</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>AG2086</t>
+          <t>AG2085</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>COSMETIC BAGS PK3 3 ASST</t>
+          <t>COSMETIC BLENDING SPONGE</t>
         </is>
       </c>
       <c r="D511" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E511" s="3" t="n">
-        <v>38243</v>
+        <v>6464</v>
       </c>
       <c r="F511" t="inlineStr">
         <is>
@@ -14652,24 +14652,24 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>9333527429797</t>
+          <t>9333527115522</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>AG2085</t>
+          <t>AG0391</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>COSMETIC BLENDING SPONGE</t>
+          <t>COSMETIC BRUSHES 3 ASST</t>
         </is>
       </c>
       <c r="D512" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E512" s="3" t="n">
-        <v>6464</v>
+        <v>15837</v>
       </c>
       <c r="F512" t="inlineStr">
         <is>
@@ -14680,24 +14680,24 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>9333527115522</t>
+          <t>9333527033208</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>AG0391</t>
+          <t>SP0055</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>COSMETIC BRUSHES 3 ASST</t>
+          <t>COPY PAPER NEON 30pk A4</t>
         </is>
       </c>
       <c r="D513" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E513" s="3" t="n">
-        <v>15837</v>
+        <v>5652</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
@@ -14806,7 +14806,7 @@
         </is>
       </c>
       <c r="D517" s="2" t="n">
-        <v>747</v>
+        <v>730</v>
       </c>
       <c r="E517" s="3" t="n">
         <v>8446</v>
@@ -17691,7 +17691,7 @@
         </is>
       </c>
       <c r="D620" s="2" t="n">
-        <v>816</v>
+        <v>792</v>
       </c>
       <c r="E620" s="3" t="n">
         <v>10114</v>
@@ -17747,7 +17747,7 @@
         </is>
       </c>
       <c r="D622" s="2" t="n">
-        <v>263</v>
+        <v>239</v>
       </c>
       <c r="E622" s="3" t="n">
         <v>9901</v>
@@ -17943,7 +17943,7 @@
         </is>
       </c>
       <c r="D629" s="2" t="n">
-        <v>3551</v>
+        <v>3419</v>
       </c>
       <c r="E629" s="3" t="n">
         <v>10251</v>
@@ -17971,7 +17971,7 @@
         </is>
       </c>
       <c r="D630" s="2" t="n">
-        <v>65</v>
+        <v>-20</v>
       </c>
       <c r="E630" s="3" t="n">
         <v>12094</v>
@@ -19091,7 +19091,7 @@
         </is>
       </c>
       <c r="D670" s="2" t="n">
-        <v>681</v>
+        <v>669</v>
       </c>
       <c r="E670" s="3" t="n">
         <v>6417</v>
@@ -19147,7 +19147,7 @@
         </is>
       </c>
       <c r="D672" s="2" t="n">
-        <v>882</v>
+        <v>866</v>
       </c>
       <c r="E672" s="3" t="n">
         <v>11078</v>
@@ -20575,7 +20575,7 @@
         </is>
       </c>
       <c r="D723" s="2" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E723" s="3" t="n">
         <v>4213</v>
@@ -21331,7 +21331,7 @@
         </is>
       </c>
       <c r="D750" s="2" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E750" s="3" t="n">
         <v>14242</v>
@@ -22591,7 +22591,7 @@
         </is>
       </c>
       <c r="D795" s="2" t="n">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="E795" s="3" t="n">
         <v>9108</v>
@@ -22619,7 +22619,7 @@
         </is>
       </c>
       <c r="D796" s="2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E796" s="3" t="n">
         <v>6934</v>
@@ -22647,7 +22647,7 @@
         </is>
       </c>
       <c r="D797" s="2" t="n">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="E797" s="3" t="n">
         <v>7465</v>
@@ -24495,7 +24495,7 @@
         </is>
       </c>
       <c r="D863" s="2" t="n">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="E863" s="3" t="n">
         <v>5764</v>
@@ -24579,7 +24579,7 @@
         </is>
       </c>
       <c r="D866" s="2" t="n">
-        <v>387</v>
+        <v>367</v>
       </c>
       <c r="E866" s="3" t="n">
         <v>7564</v>
@@ -24607,7 +24607,7 @@
         </is>
       </c>
       <c r="D867" s="2" t="n">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="E867" s="3" t="n">
         <v>12738</v>
@@ -24803,7 +24803,7 @@
         </is>
       </c>
       <c r="D874" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E874" s="3" t="n">
         <v>9239</v>
@@ -25084,7 +25084,7 @@
         </is>
       </c>
       <c r="D884" s="2" t="n">
-        <v>1034</v>
+        <v>1022</v>
       </c>
       <c r="E884" s="3" t="n">
         <v>14096</v>
@@ -25140,7 +25140,7 @@
         </is>
       </c>
       <c r="D886" s="2" t="n">
-        <v>438</v>
+        <v>423</v>
       </c>
       <c r="E886" s="3" t="n">
         <v>17750</v>
@@ -25420,7 +25420,7 @@
         </is>
       </c>
       <c r="D896" s="2" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E896" s="3" t="n">
         <v>5433</v>
@@ -25448,7 +25448,7 @@
         </is>
       </c>
       <c r="D897" s="2" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E897" s="3" t="n">
         <v>7856</v>
@@ -25476,7 +25476,7 @@
         </is>
       </c>
       <c r="D898" s="2" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E898" s="3" t="n">
         <v>5470</v>
@@ -25504,7 +25504,7 @@
         </is>
       </c>
       <c r="D899" s="2" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="E899" s="3" t="n">
         <v>7856</v>
@@ -25953,7 +25953,7 @@
         </is>
       </c>
       <c r="D915" s="2" t="n">
-        <v>1282</v>
+        <v>1256</v>
       </c>
       <c r="E915" s="3" t="n">
         <v>8181</v>
@@ -26261,7 +26261,7 @@
         </is>
       </c>
       <c r="D926" s="2" t="n">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="E926" s="3" t="n">
         <v>8988</v>
@@ -27608,7 +27608,7 @@
         </is>
       </c>
       <c r="D974" s="2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E974" s="3" t="n">
         <v>7700</v>
@@ -29932,7 +29932,7 @@
         </is>
       </c>
       <c r="D1057" s="2" t="n">
-        <v>1720</v>
+        <v>1672</v>
       </c>
       <c r="E1057" s="3" t="n">
         <v>7090</v>
@@ -30436,7 +30436,7 @@
         </is>
       </c>
       <c r="D1075" s="2" t="n">
-        <v>661</v>
+        <v>637</v>
       </c>
       <c r="E1075" s="3" t="n">
         <v>2930</v>
@@ -30604,7 +30604,7 @@
         </is>
       </c>
       <c r="D1081" s="2" t="n">
-        <v>2384</v>
+        <v>2354</v>
       </c>
       <c r="E1081" s="3" t="n">
         <v>8767</v>
@@ -31417,7 +31417,7 @@
         </is>
       </c>
       <c r="D1110" s="2" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E1110" s="3" t="n">
         <v>7008</v>
@@ -31781,7 +31781,7 @@
         </is>
       </c>
       <c r="D1123" s="2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E1123" s="3" t="n">
         <v>20164</v>
@@ -31809,7 +31809,7 @@
         </is>
       </c>
       <c r="D1124" s="2" t="n">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E1124" s="3" t="n">
         <v>19007</v>
@@ -32341,7 +32341,7 @@
         </is>
       </c>
       <c r="D1143" s="2" t="n">
-        <v>502</v>
+        <v>490</v>
       </c>
       <c r="E1143" s="3" t="n">
         <v>9226</v>
@@ -32453,7 +32453,7 @@
         </is>
       </c>
       <c r="D1147" s="2" t="n">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="E1147" s="3" t="n">
         <v>11027</v>
@@ -32845,7 +32845,7 @@
         </is>
       </c>
       <c r="D1161" s="2" t="n">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E1161" s="3" t="n">
         <v>8591</v>
@@ -37773,7 +37773,7 @@
         </is>
       </c>
       <c r="D1337" s="2" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E1337" s="3" t="n">
         <v>13998</v>
@@ -38249,7 +38249,7 @@
         </is>
       </c>
       <c r="D1354" s="2" t="n">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="E1354" s="3" t="n">
         <v>14320</v>
@@ -38277,7 +38277,7 @@
         </is>
       </c>
       <c r="D1355" s="2" t="n">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="E1355" s="3" t="n">
         <v>13595</v>
@@ -38305,7 +38305,7 @@
         </is>
       </c>
       <c r="D1356" s="2" t="n">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="E1356" s="3" t="n">
         <v>8246</v>
@@ -39565,7 +39565,7 @@
         </is>
       </c>
       <c r="D1401" s="2" t="n">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="E1401" s="3" t="n">
         <v>5674</v>
@@ -39649,7 +39649,7 @@
         </is>
       </c>
       <c r="D1404" s="2" t="n">
-        <v>679</v>
+        <v>655</v>
       </c>
       <c r="E1404" s="3" t="n">
         <v>12595</v>
@@ -39677,7 +39677,7 @@
         </is>
       </c>
       <c r="D1405" s="2" t="n">
-        <v>1438</v>
+        <v>1414</v>
       </c>
       <c r="E1405" s="3" t="n">
         <v>10295</v>
@@ -39789,7 +39789,7 @@
         </is>
       </c>
       <c r="D1409" s="2" t="n">
-        <v>713</v>
+        <v>689</v>
       </c>
       <c r="E1409" s="3" t="n">
         <v>7174</v>
@@ -40629,7 +40629,7 @@
         </is>
       </c>
       <c r="D1439" s="2" t="n">
-        <v>792</v>
+        <v>756</v>
       </c>
       <c r="E1439" s="3" t="n">
         <v>10487</v>
@@ -40713,7 +40713,7 @@
         </is>
       </c>
       <c r="D1442" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E1442" s="3" t="n">
         <v>15335</v>
@@ -41917,7 +41917,7 @@
         </is>
       </c>
       <c r="D1485" s="2" t="n">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="E1485" s="3" t="n">
         <v>11672</v>
@@ -42057,7 +42057,7 @@
         </is>
       </c>
       <c r="D1490" s="2" t="n">
-        <v>1541</v>
+        <v>1517</v>
       </c>
       <c r="E1490" s="3" t="n">
         <v>11094</v>
@@ -42085,7 +42085,7 @@
         </is>
       </c>
       <c r="D1491" s="2" t="n">
-        <v>1673</v>
+        <v>1649</v>
       </c>
       <c r="E1491" s="3" t="n">
         <v>10548</v>
@@ -42953,7 +42953,7 @@
         </is>
       </c>
       <c r="D1522" s="2" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E1522" s="3" t="n">
         <v>14636</v>
@@ -43569,7 +43569,7 @@
         </is>
       </c>
       <c r="D1544" s="2" t="n">
-        <v>273</v>
+        <v>240</v>
       </c>
       <c r="E1544" s="3" t="n">
         <v>15250</v>
@@ -43625,7 +43625,7 @@
         </is>
       </c>
       <c r="D1546" s="2" t="n">
-        <v>207</v>
+        <v>183</v>
       </c>
       <c r="E1546" s="3" t="n">
         <v>11283</v>
@@ -44073,7 +44073,7 @@
         </is>
       </c>
       <c r="D1562" s="2" t="n">
-        <v>2463</v>
+        <v>2415</v>
       </c>
       <c r="E1562" s="3" t="n">
         <v>7312</v>
@@ -44241,7 +44241,7 @@
         </is>
       </c>
       <c r="D1568" s="2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E1568" s="3" t="n">
         <v>7390</v>
@@ -45025,7 +45025,7 @@
         </is>
       </c>
       <c r="D1596" s="2" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E1596" s="3" t="n">
         <v>27542</v>
@@ -45558,7 +45558,7 @@
         </is>
       </c>
       <c r="D1615" s="2" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E1615" s="3" t="n">
         <v>17779</v>
@@ -46511,7 +46511,7 @@
         </is>
       </c>
       <c r="D1649" s="2" t="n">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="E1649" s="3" t="n">
         <v>19684</v>

</xml_diff>